<commit_message>
Updated cash sheet columns
</commit_message>
<xml_diff>
--- a/inputs/Mappings/GL_Mappings.xlsx
+++ b/inputs/Mappings/GL_Mappings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://clearwateranalytics-my.sharepoint.com/personal/matthewray_clearwateranalytics_com/Documents/Desktop/Ladder/Python/GL_Entries/inputs/Mappings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="254" documentId="8_{897F505C-C968-4279-9C81-5508E05D2B36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B6D3DBB-4D60-4A53-B021-3EA45B985DBC}"/>
+  <xr:revisionPtr revIDLastSave="255" documentId="8_{897F505C-C968-4279-9C81-5508E05D2B36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9A4CE0F-E615-4C28-B4A6-4AA1D83B0821}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B4EF2F62-3A9F-467D-A890-BA7C6F3ED471}"/>
+    <workbookView xWindow="1005" yWindow="6165" windowWidth="21600" windowHeight="12645" activeTab="1" xr2:uid="{B4EF2F62-3A9F-467D-A890-BA7C6F3ED471}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -406,6 +406,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1249,7 +1253,7 @@
   <cols>
     <col min="1" max="1" width="30.140625" customWidth="1"/>
     <col min="2" max="5" width="27.42578125" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="6" max="6" width="34.85546875" customWidth="1"/>
     <col min="7" max="7" width="13.5703125" customWidth="1"/>
     <col min="9" max="9" width="34.7109375" customWidth="1"/>
   </cols>

</xml_diff>